<commit_message>
ADD webpage. MOD language
</commit_message>
<xml_diff>
--- a/Fatture/Registro-Spese.xlsx
+++ b/Fatture/Registro-Spese.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-05 15:04:01</t>
+          <t>2026-08-09 13:45:19</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-13 — IONOS VPS Linux L+ (trainmind-vps) (69 gg)</t>
+          <t>2026-10-13 — IONOS VPS Linux L+ (trainmind-vps) (65 gg)</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>

</xml_diff>